<commit_message>
Add UPWORK and YOUTUBE to vendor lookup reference
</commit_message>
<xml_diff>
--- a/vendor_lookup_reference.xlsx
+++ b/vendor_lookup_reference.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wopi.dropbox.com/wopi/files/oid_11943546333133869312/WOPIServiceId_TP_DROPBOX_PLUS/WOPIUserId_-/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Irfan\Documents\amex-receipt-checker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B76BE6F2-5684-4088-8981-258A05F515B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{101D6C96-63A2-4A84-B67F-0D4A492E4724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Transaction Details" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2088" uniqueCount="811">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2094" uniqueCount="811">
   <si>
     <t/>
   </si>
@@ -3785,31 +3785,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V96"/>
-  <sheetFormatPr defaultColWidth="25.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="25.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.36328125" style="48" customWidth="1"/>
-    <col min="4" max="6" width="23.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.26953125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="41.90625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.81640625" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="13.54296875" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="13.54296875" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="116.453125" customWidth="1"/>
-    <col min="13" max="13" width="41.90625" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="50.90625" hidden="1" customWidth="1"/>
-    <col min="15" max="15" width="19.26953125" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="12.7265625" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="13.6328125" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="18.7265625" hidden="1" customWidth="1"/>
-    <col min="19" max="19" width="38.90625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" style="48" customWidth="1"/>
+    <col min="4" max="6" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="41.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.85546875" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5703125" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="13.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="116.42578125" customWidth="1"/>
+    <col min="13" max="13" width="41.85546875" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="50.85546875" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="19.28515625" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="13.5703125" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="18.7109375" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="38.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.140625" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="25" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="22.90625" customWidth="1"/>
+    <col min="22" max="22" width="22.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
@@ -3822,7 +3822,7 @@
       <c r="F1" s="86"/>
       <c r="G1" s="86"/>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>3</v>
       </c>
@@ -3835,7 +3835,7 @@
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
@@ -3848,7 +3848,7 @@
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>5</v>
       </c>
@@ -3861,7 +3861,7 @@
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>6</v>
       </c>
@@ -3874,7 +3874,7 @@
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
     </row>
-    <row r="6" spans="1:22" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>0</v>
       </c>
@@ -3904,7 +3904,7 @@
       </c>
       <c r="V6" s="12"/>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>7</v>
       </c>
@@ -3972,7 +3972,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" s="20" t="s">
         <v>440</v>
       </c>
@@ -4034,7 +4034,7 @@
       </c>
       <c r="V8" s="25"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" s="49" t="s">
         <v>440</v>
       </c>
@@ -4098,7 +4098,7 @@
       </c>
       <c r="V9" s="56"/>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" s="20" t="s">
         <v>440</v>
       </c>
@@ -4160,7 +4160,7 @@
       </c>
       <c r="V10" s="25"/>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" s="49" t="s">
         <v>440</v>
       </c>
@@ -4224,7 +4224,7 @@
       </c>
       <c r="V11" s="56"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" s="49" t="s">
         <v>404</v>
       </c>
@@ -4288,7 +4288,7 @@
       </c>
       <c r="V12" s="56"/>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" s="20" t="s">
         <v>404</v>
       </c>
@@ -4352,7 +4352,7 @@
       </c>
       <c r="V13" s="25"/>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" s="49" t="s">
         <v>404</v>
       </c>
@@ -4418,7 +4418,7 @@
       </c>
       <c r="V14" s="56"/>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" s="49" t="s">
         <v>404</v>
       </c>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="V15" s="56"/>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" s="20" t="s">
         <v>404</v>
       </c>
@@ -4546,7 +4546,7 @@
       </c>
       <c r="V16" s="25"/>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17" s="49" t="s">
         <v>404</v>
       </c>
@@ -4610,7 +4610,7 @@
       </c>
       <c r="V17" s="56"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A18" s="20" t="s">
         <v>404</v>
       </c>
@@ -4672,7 +4672,7 @@
       </c>
       <c r="V18" s="25"/>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19" s="20" t="s">
         <v>386</v>
       </c>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="V19" s="25"/>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A20" s="20" t="s">
         <v>386</v>
       </c>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="V20" s="25"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A21" s="20" t="s">
         <v>386</v>
       </c>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="V21" s="25"/>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
         <v>369</v>
       </c>
@@ -4922,7 +4922,7 @@
       </c>
       <c r="V22" s="25"/>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A23" s="49" t="s">
         <v>369</v>
       </c>
@@ -4988,7 +4988,7 @@
       </c>
       <c r="V23" s="56"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A24" s="49" t="s">
         <v>369</v>
       </c>
@@ -5052,7 +5052,7 @@
       </c>
       <c r="V24" s="56"/>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A25" s="49" t="s">
         <v>348</v>
       </c>
@@ -5116,7 +5116,7 @@
       </c>
       <c r="V25" s="56"/>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A26" s="20" t="s">
         <v>348</v>
       </c>
@@ -5178,7 +5178,7 @@
       </c>
       <c r="V26" s="25"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A27" s="20" t="s">
         <v>348</v>
       </c>
@@ -5240,7 +5240,7 @@
       </c>
       <c r="V27" s="25"/>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A28" s="20" t="s">
         <v>345</v>
       </c>
@@ -5304,7 +5304,7 @@
       </c>
       <c r="V28" s="25"/>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A29" s="20" t="s">
         <v>342</v>
       </c>
@@ -5368,7 +5368,7 @@
       </c>
       <c r="V29" s="25"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A30" s="20" t="s">
         <v>333</v>
       </c>
@@ -5430,7 +5430,7 @@
       </c>
       <c r="V30" s="25"/>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A31" s="20" t="s">
         <v>333</v>
       </c>
@@ -5492,7 +5492,7 @@
       </c>
       <c r="V31" s="25"/>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A32" s="20" t="s">
         <v>320</v>
       </c>
@@ -5554,7 +5554,7 @@
       </c>
       <c r="V32" s="25"/>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A33" s="49" t="s">
         <v>320</v>
       </c>
@@ -5618,7 +5618,7 @@
       </c>
       <c r="V33" s="56"/>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A34" s="20" t="s">
         <v>320</v>
       </c>
@@ -5680,7 +5680,7 @@
       </c>
       <c r="V34" s="25"/>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A35" s="49" t="s">
         <v>320</v>
       </c>
@@ -5744,7 +5744,7 @@
       </c>
       <c r="V35" s="56"/>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A36" s="20" t="s">
         <v>315</v>
       </c>
@@ -5806,7 +5806,7 @@
       </c>
       <c r="V36" s="25"/>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A37" s="49" t="s">
         <v>315</v>
       </c>
@@ -5870,7 +5870,7 @@
       </c>
       <c r="V37" s="56"/>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A38" s="20" t="s">
         <v>286</v>
       </c>
@@ -5934,7 +5934,7 @@
       </c>
       <c r="V38" s="25"/>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A39" s="20" t="s">
         <v>286</v>
       </c>
@@ -5998,7 +5998,7 @@
       </c>
       <c r="V39" s="25"/>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A40" s="20" t="s">
         <v>286</v>
       </c>
@@ -6062,7 +6062,7 @@
       </c>
       <c r="V40" s="25"/>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A41" s="20" t="s">
         <v>286</v>
       </c>
@@ -6124,7 +6124,7 @@
       </c>
       <c r="V41" s="25"/>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A42" s="49" t="s">
         <v>286</v>
       </c>
@@ -6188,7 +6188,7 @@
       </c>
       <c r="V42" s="56"/>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A43" s="20" t="s">
         <v>286</v>
       </c>
@@ -6252,7 +6252,7 @@
       </c>
       <c r="V43" s="25"/>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A44" s="20" t="s">
         <v>286</v>
       </c>
@@ -6314,7 +6314,7 @@
       </c>
       <c r="V44" s="25"/>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A45" s="20" t="s">
         <v>286</v>
       </c>
@@ -6376,7 +6376,7 @@
       </c>
       <c r="V45" s="25"/>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A46" s="20" t="s">
         <v>275</v>
       </c>
@@ -6440,7 +6440,7 @@
       </c>
       <c r="V46" s="25"/>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A47" s="20" t="s">
         <v>275</v>
       </c>
@@ -6504,7 +6504,7 @@
       </c>
       <c r="V47" s="25"/>
     </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:22" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="49" t="s">
         <v>275</v>
       </c>
@@ -6568,7 +6568,7 @@
       </c>
       <c r="V48" s="56"/>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>266</v>
       </c>
@@ -6632,7 +6632,7 @@
       </c>
       <c r="V49" s="25"/>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A50" s="49" t="s">
         <v>266</v>
       </c>
@@ -6696,7 +6696,7 @@
       </c>
       <c r="V50" s="56"/>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A51" s="20" t="s">
         <v>252</v>
       </c>
@@ -6758,7 +6758,7 @@
       </c>
       <c r="V51" s="25"/>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A52" s="49" t="s">
         <v>252</v>
       </c>
@@ -6822,7 +6822,7 @@
       </c>
       <c r="V52" s="56"/>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A53" s="49" t="s">
         <v>252</v>
       </c>
@@ -6886,7 +6886,7 @@
       </c>
       <c r="V53" s="56"/>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A54" s="20" t="s">
         <v>228</v>
       </c>
@@ -6948,7 +6948,7 @@
       </c>
       <c r="V54" s="25"/>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A55" s="20" t="s">
         <v>228</v>
       </c>
@@ -7010,7 +7010,7 @@
       </c>
       <c r="V55" s="25"/>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A56" s="20" t="s">
         <v>228</v>
       </c>
@@ -7072,7 +7072,7 @@
       </c>
       <c r="V56" s="25"/>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A57" s="20" t="s">
         <v>228</v>
       </c>
@@ -7134,7 +7134,7 @@
       </c>
       <c r="V57" s="25"/>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A58" s="49" t="s">
         <v>228</v>
       </c>
@@ -7198,7 +7198,7 @@
       </c>
       <c r="V58" s="56"/>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A59" s="20" t="s">
         <v>185</v>
       </c>
@@ -7260,7 +7260,7 @@
       </c>
       <c r="V59" s="25"/>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A60" s="20" t="s">
         <v>185</v>
       </c>
@@ -7322,7 +7322,7 @@
       </c>
       <c r="V60" s="25"/>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A61" s="20" t="s">
         <v>185</v>
       </c>
@@ -7384,7 +7384,7 @@
       </c>
       <c r="V61" s="25"/>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A62" s="49" t="s">
         <v>185</v>
       </c>
@@ -7450,7 +7450,7 @@
       </c>
       <c r="V62" s="56"/>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A63" s="20" t="s">
         <v>185</v>
       </c>
@@ -7514,7 +7514,7 @@
       </c>
       <c r="V63" s="25"/>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A64" s="20" t="s">
         <v>185</v>
       </c>
@@ -7576,7 +7576,7 @@
       </c>
       <c r="V64" s="25"/>
     </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A65" s="49" t="s">
         <v>185</v>
       </c>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="V65" s="56"/>
     </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A66" s="49" t="s">
         <v>185</v>
       </c>
@@ -7704,7 +7704,7 @@
       </c>
       <c r="V66" s="56"/>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A67" s="20" t="s">
         <v>173</v>
       </c>
@@ -7768,7 +7768,7 @@
       </c>
       <c r="V67" s="25"/>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A68" s="20" t="s">
         <v>173</v>
       </c>
@@ -7832,7 +7832,7 @@
       </c>
       <c r="V68" s="25"/>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A69" s="20" t="s">
         <v>173</v>
       </c>
@@ -7894,7 +7894,7 @@
       </c>
       <c r="V69" s="25"/>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A70" s="20" t="s">
         <v>161</v>
       </c>
@@ -7956,7 +7956,7 @@
       </c>
       <c r="V70" s="25"/>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A71" s="20" t="s">
         <v>161</v>
       </c>
@@ -8018,7 +8018,7 @@
       </c>
       <c r="V71" s="25"/>
     </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A72" s="20" t="s">
         <v>156</v>
       </c>
@@ -8082,7 +8082,7 @@
       </c>
       <c r="V72" s="25"/>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A73" s="20" t="s">
         <v>156</v>
       </c>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="V73" s="25"/>
     </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A74" s="20" t="s">
         <v>147</v>
       </c>
@@ -8208,7 +8208,7 @@
       </c>
       <c r="V74" s="25"/>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A75" s="20" t="s">
         <v>147</v>
       </c>
@@ -8270,7 +8270,7 @@
       </c>
       <c r="V75" s="25"/>
     </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A76" s="20" t="s">
         <v>139</v>
       </c>
@@ -8334,7 +8334,7 @@
       </c>
       <c r="V76" s="25"/>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A77" s="20" t="s">
         <v>139</v>
       </c>
@@ -8398,7 +8398,7 @@
       </c>
       <c r="V77" s="25"/>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A78" s="20" t="s">
         <v>132</v>
       </c>
@@ -8460,7 +8460,7 @@
       </c>
       <c r="V78" s="25"/>
     </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A79" s="20" t="s">
         <v>125</v>
       </c>
@@ -8524,7 +8524,7 @@
       </c>
       <c r="V79" s="25"/>
     </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A80" s="20" t="s">
         <v>103</v>
       </c>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="V80" s="25"/>
     </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A81" s="20" t="s">
         <v>103</v>
       </c>
@@ -8644,7 +8644,7 @@
         <v>737</v>
       </c>
     </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A82" s="20" t="s">
         <v>103</v>
       </c>
@@ -8702,7 +8702,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A83" s="20" t="s">
         <v>86</v>
       </c>
@@ -8764,7 +8764,7 @@
       </c>
       <c r="V83" s="25"/>
     </row>
-    <row r="84" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A84" s="20" t="s">
         <v>86</v>
       </c>
@@ -8826,7 +8826,7 @@
       </c>
       <c r="V84" s="25"/>
     </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A85" s="20" t="s">
         <v>86</v>
       </c>
@@ -8884,7 +8884,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A86" s="20" t="s">
         <v>78</v>
       </c>
@@ -8946,7 +8946,7 @@
       </c>
       <c r="V86" s="25"/>
     </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A87" s="20" t="s">
         <v>57</v>
       </c>
@@ -9010,7 +9010,7 @@
       </c>
       <c r="V87" s="25"/>
     </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A88" s="20" t="s">
         <v>57</v>
       </c>
@@ -9072,7 +9072,7 @@
       </c>
       <c r="V88" s="25"/>
     </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A89" s="20" t="s">
         <v>57</v>
       </c>
@@ -9134,7 +9134,7 @@
       </c>
       <c r="V89" s="25"/>
     </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A90" s="20" t="s">
         <v>50</v>
       </c>
@@ -9196,7 +9196,7 @@
       </c>
       <c r="V90" s="25"/>
     </row>
-    <row r="91" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A91" s="20" t="s">
         <v>32</v>
       </c>
@@ -9260,7 +9260,7 @@
       </c>
       <c r="V91" s="25"/>
     </row>
-    <row r="92" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A92" s="20" t="s">
         <v>32</v>
       </c>
@@ -9324,7 +9324,7 @@
       </c>
       <c r="V92" s="25"/>
     </row>
-    <row r="93" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A93" s="49" t="s">
         <v>32</v>
       </c>
@@ -9388,7 +9388,7 @@
       </c>
       <c r="V93" s="56"/>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A94" s="20" t="s">
         <v>21</v>
       </c>
@@ -9450,8 +9450,8 @@
       </c>
       <c r="V94" s="25"/>
     </row>
-    <row r="95" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="96" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="96" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="J96" s="1" t="s">
         <v>459</v>
       </c>
@@ -9477,16 +9477,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8E0AB0-A30D-4D7D-84FD-A751B73043A8}">
   <dimension ref="A1:D85"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.36328125" style="15" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="40.36328125" style="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="47.36328125" style="15" customWidth="1"/>
+    <col min="1" max="1" width="13.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="47.42578125" style="15" customWidth="1"/>
     <col min="4" max="4" width="26" style="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.7265625" style="15"/>
+    <col min="5" max="16384" width="8.7109375" style="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
         <v>469</v>
       </c>
@@ -9497,7 +9497,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
         <v>471</v>
       </c>
@@ -9511,7 +9511,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
         <v>475</v>
       </c>
@@ -9519,7 +9519,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
         <v>477</v>
       </c>
@@ -9527,7 +9527,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
         <v>479</v>
       </c>
@@ -9535,7 +9535,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
         <v>481</v>
       </c>
@@ -9543,7 +9543,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
         <v>483</v>
       </c>
@@ -9551,11 +9551,11 @@
         <v>484</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="16"/>
       <c r="B8" s="16"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
         <v>485</v>
       </c>
@@ -9566,7 +9566,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="16" t="s">
         <v>488</v>
       </c>
@@ -9574,7 +9574,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
         <v>490</v>
       </c>
@@ -9582,7 +9582,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
         <v>492</v>
       </c>
@@ -9590,11 +9590,11 @@
         <v>493</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="16"/>
       <c r="B13" s="16"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="16" t="s">
         <v>494</v>
       </c>
@@ -9608,7 +9608,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="16" t="s">
         <v>498</v>
       </c>
@@ -9616,7 +9616,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="s">
         <v>500</v>
       </c>
@@ -9624,7 +9624,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
         <v>502</v>
       </c>
@@ -9632,7 +9632,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
         <v>504</v>
       </c>
@@ -9640,7 +9640,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
         <v>506</v>
       </c>
@@ -9648,7 +9648,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
         <v>508</v>
       </c>
@@ -9656,7 +9656,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="16" t="s">
         <v>510</v>
       </c>
@@ -9664,7 +9664,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="16" t="s">
         <v>512</v>
       </c>
@@ -9672,7 +9672,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
         <v>514</v>
       </c>
@@ -9680,11 +9680,11 @@
         <v>515</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="16"/>
       <c r="B24" s="16"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="16" t="s">
         <v>516</v>
       </c>
@@ -9695,7 +9695,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="16" t="s">
         <v>519</v>
       </c>
@@ -9703,7 +9703,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="18" t="s">
         <v>521</v>
       </c>
@@ -9711,7 +9711,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="16" t="s">
         <v>523</v>
       </c>
@@ -9719,11 +9719,11 @@
         <v>524</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="16"/>
       <c r="B29" s="16"/>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="17" t="s">
         <v>525</v>
       </c>
@@ -9737,7 +9737,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="17" t="s">
         <v>529</v>
       </c>
@@ -9745,7 +9745,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="16" t="s">
         <v>531</v>
       </c>
@@ -9753,7 +9753,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="16" t="s">
         <v>533</v>
       </c>
@@ -9761,7 +9761,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="16" t="s">
         <v>535</v>
       </c>
@@ -9769,7 +9769,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="16" t="s">
         <v>537</v>
       </c>
@@ -9777,7 +9777,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="16" t="s">
         <v>539</v>
       </c>
@@ -9785,7 +9785,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="17" t="s">
         <v>541</v>
       </c>
@@ -9796,7 +9796,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="16" t="s">
         <v>544</v>
       </c>
@@ -9807,7 +9807,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="16" t="s">
         <v>547</v>
       </c>
@@ -9815,7 +9815,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="16" t="s">
         <v>549</v>
       </c>
@@ -9823,7 +9823,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="16" t="s">
         <v>551</v>
       </c>
@@ -9831,7 +9831,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="17" t="s">
         <v>553</v>
       </c>
@@ -9839,7 +9839,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="17" t="s">
         <v>555</v>
       </c>
@@ -9847,7 +9847,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="17" t="s">
         <v>557</v>
       </c>
@@ -9855,7 +9855,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="16" t="s">
         <v>559</v>
       </c>
@@ -9863,7 +9863,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="17" t="s">
         <v>561</v>
       </c>
@@ -9871,7 +9871,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="17" t="s">
         <v>563</v>
       </c>
@@ -9879,7 +9879,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="17" t="s">
         <v>565</v>
       </c>
@@ -9887,7 +9887,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="16" t="s">
         <v>567</v>
       </c>
@@ -9898,7 +9898,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="16" t="s">
         <v>570</v>
       </c>
@@ -9906,7 +9906,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="16" t="s">
         <v>572</v>
       </c>
@@ -9914,7 +9914,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="16" t="s">
         <v>574</v>
       </c>
@@ -9922,7 +9922,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="16" t="s">
         <v>576</v>
       </c>
@@ -9930,7 +9930,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="16" t="s">
         <v>578</v>
       </c>
@@ -9938,7 +9938,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="17" t="s">
         <v>580</v>
       </c>
@@ -9946,11 +9946,11 @@
         <v>581</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="16"/>
       <c r="B56" s="16"/>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="16" t="s">
         <v>582</v>
       </c>
@@ -9961,7 +9961,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="16" t="s">
         <v>585</v>
       </c>
@@ -9969,7 +9969,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="16" t="s">
         <v>587</v>
       </c>
@@ -9977,7 +9977,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="16" t="s">
         <v>589</v>
       </c>
@@ -9985,11 +9985,11 @@
         <v>590</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="16"/>
       <c r="B61" s="16"/>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="16" t="s">
         <v>591</v>
       </c>
@@ -10000,7 +10000,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="16" t="s">
         <v>594</v>
       </c>
@@ -10008,7 +10008,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="16" t="s">
         <v>596</v>
       </c>
@@ -10016,7 +10016,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="16" t="s">
         <v>598</v>
       </c>
@@ -10024,11 +10024,11 @@
         <v>599</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="16"/>
       <c r="B66" s="16"/>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="16" t="s">
         <v>600</v>
       </c>
@@ -10039,7 +10039,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="16" t="s">
         <v>603</v>
       </c>
@@ -10047,7 +10047,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="16" t="s">
         <v>605</v>
       </c>
@@ -10055,7 +10055,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="16" t="s">
         <v>607</v>
       </c>
@@ -10063,7 +10063,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="16" t="s">
         <v>609</v>
       </c>
@@ -10071,7 +10071,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" s="16" t="s">
         <v>611</v>
       </c>
@@ -10079,7 +10079,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="16" t="s">
         <v>613</v>
       </c>
@@ -10087,7 +10087,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="16" t="s">
         <v>615</v>
       </c>
@@ -10095,7 +10095,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" s="16" t="s">
         <v>617</v>
       </c>
@@ -10106,7 +10106,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="16" t="s">
         <v>620</v>
       </c>
@@ -10117,7 +10117,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" s="16" t="s">
         <v>623</v>
       </c>
@@ -10125,11 +10125,11 @@
         <v>624</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="16"/>
       <c r="B78" s="16"/>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" s="16" t="s">
         <v>625</v>
       </c>
@@ -10140,7 +10140,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" s="16" t="s">
         <v>628</v>
       </c>
@@ -10148,7 +10148,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="16" t="s">
         <v>630</v>
       </c>
@@ -10156,7 +10156,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" s="16" t="s">
         <v>632</v>
       </c>
@@ -10164,7 +10164,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" s="16" t="s">
         <v>634</v>
       </c>
@@ -10172,7 +10172,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" s="15" t="s">
         <v>636</v>
       </c>
@@ -10193,18 +10193,18 @@
   <sheetPr>
     <tabColor theme="4" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="B2:E90"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="B2:E92"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.81640625" style="70"/>
-    <col min="2" max="2" width="34.453125" style="70" customWidth="1"/>
-    <col min="3" max="3" width="12.54296875" style="70" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.54296875" style="70" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.453125" style="70" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.81640625" style="70"/>
+    <col min="1" max="1" width="8.85546875" style="70"/>
+    <col min="2" max="2" width="34.42578125" style="70" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" style="70" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.5703125" style="70" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" style="70" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.85546875" style="70"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B2" s="69" t="s">
         <v>740</v>
       </c>
@@ -10218,7 +10218,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B3" s="71" t="s">
         <v>743</v>
       </c>
@@ -10230,7 +10230,7 @@
       </c>
       <c r="E3" s="22"/>
     </row>
-    <row r="4" spans="2:5" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="71" t="s">
         <v>744</v>
       </c>
@@ -10242,7 +10242,7 @@
       </c>
       <c r="E4" s="22"/>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B5" s="71" t="s">
         <v>745</v>
       </c>
@@ -10254,7 +10254,7 @@
       </c>
       <c r="E5" s="22"/>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B6" s="32" t="s">
         <v>746</v>
       </c>
@@ -10266,7 +10266,7 @@
       </c>
       <c r="E6" s="22"/>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" s="71" t="s">
         <v>747</v>
       </c>
@@ -10278,7 +10278,7 @@
       </c>
       <c r="E7" s="22"/>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B8" s="71" t="s">
         <v>748</v>
       </c>
@@ -10290,7 +10290,7 @@
       </c>
       <c r="E8" s="22"/>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" s="71" t="s">
         <v>749</v>
       </c>
@@ -10302,7 +10302,7 @@
       </c>
       <c r="E9" s="22"/>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B10" s="71" t="s">
         <v>750</v>
       </c>
@@ -10314,7 +10314,7 @@
       </c>
       <c r="E10" s="22"/>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B11" s="71" t="s">
         <v>751</v>
       </c>
@@ -10326,7 +10326,7 @@
       </c>
       <c r="E11" s="22"/>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B12" s="71" t="s">
         <v>651</v>
       </c>
@@ -10338,7 +10338,7 @@
       </c>
       <c r="E12" s="22"/>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B13" s="71" t="s">
         <v>725</v>
       </c>
@@ -10350,7 +10350,7 @@
       </c>
       <c r="E13" s="22"/>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B14" s="71" t="s">
         <v>752</v>
       </c>
@@ -10362,7 +10362,7 @@
       </c>
       <c r="E14" s="22"/>
     </row>
-    <row r="15" spans="2:5" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="71" t="s">
         <v>753</v>
       </c>
@@ -10374,7 +10374,7 @@
       </c>
       <c r="E15" s="22"/>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B16" s="71" t="s">
         <v>727</v>
       </c>
@@ -10386,7 +10386,7 @@
       </c>
       <c r="E16" s="22"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="71" t="s">
         <v>754</v>
       </c>
@@ -10398,7 +10398,7 @@
       </c>
       <c r="E17" s="22"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18" s="71" t="s">
         <v>755</v>
       </c>
@@ -10410,7 +10410,7 @@
       </c>
       <c r="E18" s="22"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" s="71" t="s">
         <v>726</v>
       </c>
@@ -10422,7 +10422,7 @@
       </c>
       <c r="E19" s="22"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20" s="71" t="s">
         <v>681</v>
       </c>
@@ -10434,7 +10434,7 @@
       </c>
       <c r="E20" s="22"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B21" s="71" t="s">
         <v>756</v>
       </c>
@@ -10446,7 +10446,7 @@
       </c>
       <c r="E21" s="22"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22" s="71" t="s">
         <v>757</v>
       </c>
@@ -10458,7 +10458,7 @@
       </c>
       <c r="E22" s="22"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23" s="71" t="s">
         <v>722</v>
       </c>
@@ -10470,7 +10470,7 @@
       </c>
       <c r="E23" s="22"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24" s="71" t="s">
         <v>758</v>
       </c>
@@ -10482,7 +10482,7 @@
       </c>
       <c r="E24" s="22"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25" s="71" t="s">
         <v>759</v>
       </c>
@@ -10494,7 +10494,7 @@
       </c>
       <c r="E25" s="22"/>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B26" s="71" t="s">
         <v>760</v>
       </c>
@@ -10506,7 +10506,7 @@
       </c>
       <c r="E26" s="22"/>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B27" s="71" t="s">
         <v>761</v>
       </c>
@@ -10518,7 +10518,7 @@
       </c>
       <c r="E27" s="22"/>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B28" s="71" t="s">
         <v>699</v>
       </c>
@@ -10530,7 +10530,7 @@
       </c>
       <c r="E28" s="22"/>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B29" s="71" t="s">
         <v>762</v>
       </c>
@@ -10542,7 +10542,7 @@
       </c>
       <c r="E29" s="22"/>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B30" s="71" t="s">
         <v>763</v>
       </c>
@@ -10554,7 +10554,7 @@
       </c>
       <c r="E30" s="22"/>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B31" s="23" t="s">
         <v>764</v>
       </c>
@@ -10566,7 +10566,7 @@
       </c>
       <c r="E31" s="22"/>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B32" s="71" t="s">
         <v>715</v>
       </c>
@@ -10578,7 +10578,7 @@
       </c>
       <c r="E32" s="22"/>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B33" s="71" t="s">
         <v>765</v>
       </c>
@@ -10590,7 +10590,7 @@
       </c>
       <c r="E33" s="22"/>
     </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B34" s="71" t="s">
         <v>766</v>
       </c>
@@ -10602,7 +10602,7 @@
       </c>
       <c r="E34" s="22"/>
     </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B35" s="71" t="s">
         <v>767</v>
       </c>
@@ -10614,7 +10614,7 @@
       </c>
       <c r="E35" s="22"/>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B36" s="71" t="s">
         <v>705</v>
       </c>
@@ -10626,7 +10626,7 @@
       </c>
       <c r="E36" s="22"/>
     </row>
-    <row r="37" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B37" s="71" t="s">
         <v>707</v>
       </c>
@@ -10638,7 +10638,7 @@
       </c>
       <c r="E37" s="22"/>
     </row>
-    <row r="38" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B38" s="23" t="s">
         <v>709</v>
       </c>
@@ -10650,7 +10650,7 @@
       </c>
       <c r="E38" s="22"/>
     </row>
-    <row r="39" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B39" s="71" t="s">
         <v>768</v>
       </c>
@@ -10662,7 +10662,7 @@
       </c>
       <c r="E39" s="22"/>
     </row>
-    <row r="40" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B40" s="71" t="s">
         <v>704</v>
       </c>
@@ -10674,7 +10674,7 @@
       </c>
       <c r="E40" s="22"/>
     </row>
-    <row r="41" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B41" s="71" t="s">
         <v>769</v>
       </c>
@@ -10686,7 +10686,7 @@
       </c>
       <c r="E41" s="22"/>
     </row>
-    <row r="42" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B42" s="71" t="s">
         <v>770</v>
       </c>
@@ -10698,7 +10698,7 @@
       </c>
       <c r="E42" s="22"/>
     </row>
-    <row r="43" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B43" s="23" t="s">
         <v>771</v>
       </c>
@@ -10710,7 +10710,7 @@
       </c>
       <c r="E43" s="22"/>
     </row>
-    <row r="44" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B44" s="71" t="s">
         <v>772</v>
       </c>
@@ -10722,7 +10722,7 @@
       </c>
       <c r="E44" s="22"/>
     </row>
-    <row r="45" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B45" s="71" t="s">
         <v>773</v>
       </c>
@@ -10734,7 +10734,7 @@
       </c>
       <c r="E45" s="22"/>
     </row>
-    <row r="46" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B46" s="71" t="s">
         <v>774</v>
       </c>
@@ -10746,7 +10746,7 @@
       </c>
       <c r="E46" s="22"/>
     </row>
-    <row r="47" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B47" s="71" t="s">
         <v>775</v>
       </c>
@@ -10758,7 +10758,7 @@
       </c>
       <c r="E47" s="22"/>
     </row>
-    <row r="48" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B48" s="71" t="s">
         <v>776</v>
       </c>
@@ -10770,7 +10770,7 @@
       </c>
       <c r="E48" s="22"/>
     </row>
-    <row r="49" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B49" s="71" t="s">
         <v>697</v>
       </c>
@@ -10782,7 +10782,7 @@
       </c>
       <c r="E49" s="22"/>
     </row>
-    <row r="50" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B50" s="71" t="s">
         <v>777</v>
       </c>
@@ -10794,7 +10794,7 @@
       </c>
       <c r="E50" s="22"/>
     </row>
-    <row r="51" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B51" s="71" t="s">
         <v>650</v>
       </c>
@@ -10806,7 +10806,7 @@
       </c>
       <c r="E51" s="22"/>
     </row>
-    <row r="52" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B52" s="71" t="s">
         <v>778</v>
       </c>
@@ -10818,7 +10818,7 @@
       </c>
       <c r="E52" s="22"/>
     </row>
-    <row r="53" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B53" s="79" t="s">
         <v>779</v>
       </c>
@@ -10830,7 +10830,7 @@
       </c>
       <c r="E53" s="22"/>
     </row>
-    <row r="54" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B54" s="71" t="s">
         <v>780</v>
       </c>
@@ -10842,7 +10842,7 @@
       </c>
       <c r="E54" s="22"/>
     </row>
-    <row r="55" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B55" s="71" t="s">
         <v>781</v>
       </c>
@@ -10854,7 +10854,7 @@
       </c>
       <c r="E55" s="22"/>
     </row>
-    <row r="56" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B56" s="71" t="s">
         <v>782</v>
       </c>
@@ -10866,7 +10866,7 @@
       </c>
       <c r="E56" s="22"/>
     </row>
-    <row r="57" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B57" s="71" t="s">
         <v>783</v>
       </c>
@@ -10878,7 +10878,7 @@
       </c>
       <c r="E57" s="22"/>
     </row>
-    <row r="58" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B58" s="71" t="s">
         <v>784</v>
       </c>
@@ -10890,7 +10890,7 @@
       </c>
       <c r="E58" s="22"/>
     </row>
-    <row r="59" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B59" s="71" t="s">
         <v>686</v>
       </c>
@@ -10902,7 +10902,7 @@
       </c>
       <c r="E59" s="22"/>
     </row>
-    <row r="60" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B60" s="71" t="s">
         <v>785</v>
       </c>
@@ -10914,7 +10914,7 @@
       </c>
       <c r="E60" s="22"/>
     </row>
-    <row r="61" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B61" s="71" t="s">
         <v>786</v>
       </c>
@@ -10926,7 +10926,7 @@
       </c>
       <c r="E61" s="22"/>
     </row>
-    <row r="62" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B62" s="71" t="s">
         <v>787</v>
       </c>
@@ -10938,7 +10938,7 @@
       </c>
       <c r="E62" s="22"/>
     </row>
-    <row r="63" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B63" s="71" t="s">
         <v>788</v>
       </c>
@@ -10950,7 +10950,7 @@
       </c>
       <c r="E63" s="22"/>
     </row>
-    <row r="64" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B64" s="71" t="s">
         <v>789</v>
       </c>
@@ -10962,7 +10962,7 @@
       </c>
       <c r="E64" s="22"/>
     </row>
-    <row r="65" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B65" s="71" t="s">
         <v>790</v>
       </c>
@@ -10974,7 +10974,7 @@
       </c>
       <c r="E65" s="22"/>
     </row>
-    <row r="66" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B66" s="23" t="s">
         <v>791</v>
       </c>
@@ -10986,7 +10986,7 @@
       </c>
       <c r="E66" s="22"/>
     </row>
-    <row r="67" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B67" s="71" t="s">
         <v>694</v>
       </c>
@@ -10998,7 +10998,7 @@
       </c>
       <c r="E67" s="22"/>
     </row>
-    <row r="68" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B68" s="71" t="s">
         <v>792</v>
       </c>
@@ -11010,7 +11010,7 @@
       </c>
       <c r="E68" s="22"/>
     </row>
-    <row r="69" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B69" s="71" t="s">
         <v>793</v>
       </c>
@@ -11022,7 +11022,7 @@
       </c>
       <c r="E69" s="22"/>
     </row>
-    <row r="70" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B70" s="71" t="s">
         <v>717</v>
       </c>
@@ -11034,7 +11034,7 @@
       </c>
       <c r="E70" s="22"/>
     </row>
-    <row r="71" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B71" s="71" t="s">
         <v>794</v>
       </c>
@@ -11046,7 +11046,7 @@
       </c>
       <c r="E71" s="22"/>
     </row>
-    <row r="72" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B72" s="71" t="s">
         <v>795</v>
       </c>
@@ -11058,7 +11058,7 @@
       </c>
       <c r="E72" s="22"/>
     </row>
-    <row r="73" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B73" s="71" t="s">
         <v>796</v>
       </c>
@@ -11070,7 +11070,7 @@
       </c>
       <c r="E73" s="22"/>
     </row>
-    <row r="74" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B74" s="71" t="s">
         <v>665</v>
       </c>
@@ -11082,7 +11082,7 @@
       </c>
       <c r="E74" s="22"/>
     </row>
-    <row r="75" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B75" s="71" t="s">
         <v>797</v>
       </c>
@@ -11094,7 +11094,7 @@
       </c>
       <c r="E75" s="22"/>
     </row>
-    <row r="76" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B76" s="71" t="s">
         <v>798</v>
       </c>
@@ -11106,7 +11106,7 @@
       </c>
       <c r="E76" s="22"/>
     </row>
-    <row r="77" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B77" s="71" t="s">
         <v>799</v>
       </c>
@@ -11118,7 +11118,7 @@
       </c>
       <c r="E77" s="22"/>
     </row>
-    <row r="78" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B78" s="71" t="s">
         <v>673</v>
       </c>
@@ -11130,7 +11130,7 @@
       </c>
       <c r="E78" s="22"/>
     </row>
-    <row r="79" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B79" s="71" t="s">
         <v>800</v>
       </c>
@@ -11142,7 +11142,7 @@
       </c>
       <c r="E79" s="22"/>
     </row>
-    <row r="80" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B80" s="71" t="s">
         <v>671</v>
       </c>
@@ -11154,7 +11154,7 @@
       </c>
       <c r="E80" s="22"/>
     </row>
-    <row r="81" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B81" s="71" t="s">
         <v>801</v>
       </c>
@@ -11166,7 +11166,7 @@
       </c>
       <c r="E81" s="22"/>
     </row>
-    <row r="82" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B82" s="71" t="s">
         <v>802</v>
       </c>
@@ -11178,7 +11178,7 @@
       </c>
       <c r="E82" s="22"/>
     </row>
-    <row r="83" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B83" s="71" t="s">
         <v>675</v>
       </c>
@@ -11190,7 +11190,7 @@
       </c>
       <c r="E83" s="22"/>
     </row>
-    <row r="84" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B84" s="23" t="s">
         <v>803</v>
       </c>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="E84" s="22"/>
     </row>
-    <row r="85" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B85" s="23" t="s">
         <v>804</v>
       </c>
@@ -11214,7 +11214,7 @@
       </c>
       <c r="E85" s="22"/>
     </row>
-    <row r="86" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B86" s="23" t="s">
         <v>805</v>
       </c>
@@ -11226,7 +11226,7 @@
       </c>
       <c r="E86" s="22"/>
     </row>
-    <row r="87" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B87" s="22" t="s">
         <v>806</v>
       </c>
@@ -11236,7 +11236,7 @@
         <v>807</v>
       </c>
     </row>
-    <row r="88" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B88" s="32" t="s">
         <v>808</v>
       </c>
@@ -11247,7 +11247,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="89" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B89" s="32" t="s">
         <v>809</v>
       </c>
@@ -11258,7 +11258,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="90" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B90" s="82" t="s">
         <v>810</v>
       </c>
@@ -11269,16 +11269,38 @@
         <v>536</v>
       </c>
     </row>
+    <row r="91" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B91" t="s">
+        <v>667</v>
+      </c>
+      <c r="C91" s="81" t="s">
+        <v>535</v>
+      </c>
+      <c r="D91" s="81" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="92" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B92" s="32" t="s">
+        <v>706</v>
+      </c>
+      <c r="C92" s="81" t="s">
+        <v>553</v>
+      </c>
+      <c r="D92" s="81" t="s">
+        <v>554</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="B2:E2" xr:uid="{262952A2-B7A9-455F-8A76-999BAE31492A}"/>
-  <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+  <conditionalFormatting sqref="B1:B90 B92:B1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B37 B39:B42 B44:B83">
-    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>